<commit_message>
loading data in date add
</commit_message>
<xml_diff>
--- a/public/file/loading.xlsx
+++ b/public/file/loading.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t xml:space="preserve">delivery_date</t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t xml:space="preserve">pallet_number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">date</t>
   </si>
 </sst>
 </file>
@@ -59,7 +62,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -86,11 +89,6 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -135,7 +133,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -145,10 +143,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -169,10 +163,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.04"/>
@@ -195,10 +189,10 @@
       <c r="D1" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="0" t="s">
@@ -212,6 +206,9 @@
       </c>
       <c r="J1" s="0" t="s">
         <v>9</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>